<commit_message>
Updated commit before removing files and redundancies
</commit_message>
<xml_diff>
--- a/dataAcquisition/Motec_MP/plottingRequest/E07_TSV/PR_E07TSV_plotRequest.xlsx
+++ b/dataAcquisition/Motec_MP/plottingRequest/E07_TSV/PR_E07TSV_plotRequest.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SimEnv\dataAcquisition\Motec_MP\plottingRequest\E07_TSV\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SimEnv\dataAcquisition\Motec_MP\plottingRequest\E07_TSV\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7C9186E-ABF5-4145-8E36-BA1A61FC3DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC82C615-3021-487C-BC01-49098418194E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{98CBB8D2-373D-4831-8E1A-176399598E12}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{98CBB8D2-373D-4831-8E1A-176399598E12}"/>
   </bookViews>
   <sheets>
     <sheet name="plotting" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1047" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1060" uniqueCount="182">
   <si>
     <t>mathFunction</t>
   </si>
@@ -468,12 +468,6 @@
     <t>[100, 300]</t>
   </si>
   <si>
-    <t>[-20, 10]</t>
-  </si>
-  <si>
-    <t>[0, 40]</t>
-  </si>
-  <si>
     <t>trace_scatter_all</t>
   </si>
   <si>
@@ -489,15 +483,6 @@
     <t xml:space="preserve">ADR_Acceleration_Y              </t>
   </si>
   <si>
-    <t>[5,35]</t>
-  </si>
-  <si>
-    <t>[20,50]</t>
-  </si>
-  <si>
-    <t>20,50]</t>
-  </si>
-  <si>
     <t>GG</t>
   </si>
   <si>
@@ -589,6 +574,15 @@
   </si>
   <si>
     <t>Lift And Coast Time</t>
+  </si>
+  <si>
+    <t>[0, 60]</t>
+  </si>
+  <si>
+    <t>Rotation_Limited_Time</t>
+  </si>
+  <si>
+    <t>Rotation Limited Time</t>
   </si>
 </sst>
 </file>
@@ -778,7 +772,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$C$66" spid="_x0000_s1057"/>
+                  <a14:cameraTool cellRange="$C$66" spid="_x0000_s1089"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -843,7 +837,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$D$66" spid="_x0000_s1058"/>
+                  <a14:cameraTool cellRange="$D$66" spid="_x0000_s1090"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -903,13 +897,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$C$66" spid="_x0000_s1059"/>
+                  <a14:cameraTool cellRange="$C$66" spid="_x0000_s1091"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -963,13 +957,13 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$D$66" spid="_x0000_s1060"/>
+                  <a14:cameraTool cellRange="$D$66" spid="_x0000_s1092"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
           <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
             <a:srcRect/>
             <a:stretch>
               <a:fillRect/>
@@ -979,6 +973,246 @@
             <a:xfrm>
               <a:off x="4981222" y="12107333"/>
               <a:ext cx="1452739" cy="189795"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>67</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1004429" cy="193040"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="6" name="Picture 5">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9622680-ACE8-49D7-82D2-F2CED1AE6D16}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="$C$66" spid="_x0000_s1093"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="3845278" y="12573000"/>
+              <a:ext cx="1004429" cy="193040"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>67</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1413651" cy="193040"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="7" name="Picture 6">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F46F34E5-D2A9-467A-99E5-54021F90DE95}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="$D$66" spid="_x0000_s1094"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="4847167" y="12573000"/>
+              <a:ext cx="1413651" cy="193040"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>2</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>68</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1001889" cy="190500"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="8" name="Picture 7">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3A395CEB-91C7-42D8-9D42-4E160BBCA568}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="$C$66" spid="_x0000_s1095"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="3845278" y="12954000"/>
+              <a:ext cx="1001889" cy="190500"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:extLst>
+              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+                <a14:hiddenFill>
+                  <a:solidFill>
+                    <a:srgbClr val="FFFFFF"/>
+                  </a:solidFill>
+                </a14:hiddenFill>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:pic>
+        <xdr:clientData/>
+      </xdr:oneCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:oneCellAnchor>
+        <xdr:from>
+          <xdr:col>3</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>68</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:ext cx="1411111" cy="190500"/>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="9" name="Picture 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D60CEEE9-181A-43CC-A562-7AFE419FF9BD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr>
+              <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+              <a:extLst>
+                <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
+                  <a14:cameraTool cellRange="$D$66" spid="_x0000_s1096"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPicPr>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+            <a:srcRect/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="4847167" y="12954000"/>
+              <a:ext cx="1411111" cy="190500"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -1320,35 +1554,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE8B1EEC-F5CB-4522-AB96-C6BC3CAD72FB}">
-  <dimension ref="A1:AC68"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AC69"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="1" max="1" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.109375" customWidth="1"/>
-    <col min="5" max="5" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.109375" customWidth="1"/>
-    <col min="12" max="12" width="18.109375" customWidth="1"/>
-    <col min="13" max="13" width="20.109375" customWidth="1"/>
-    <col min="14" max="14" width="44.44140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.140625" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" customWidth="1"/>
+    <col min="14" max="14" width="44.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="10" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="28.109375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="25.109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="24" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="25.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="3" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1437,7 +1670,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
         <v>30</v>
       </c>
@@ -1482,7 +1715,7 @@
         <v>1</v>
       </c>
       <c r="P2" s="12" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="Q2" s="12" t="s">
         <v>41</v>
@@ -1508,7 +1741,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
         <v>35</v>
       </c>
@@ -1554,7 +1787,7 @@
         <v>1</v>
       </c>
       <c r="P3" s="12" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="Q3" s="12" t="s">
         <v>42</v>
@@ -1580,7 +1813,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
         <v>37</v>
       </c>
@@ -1626,7 +1859,7 @@
         <v>1</v>
       </c>
       <c r="P4" s="12" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="Q4" s="12" t="s">
         <v>43</v>
@@ -1652,9 +1885,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="12" t="s">
@@ -1698,7 +1931,7 @@
         <v>1</v>
       </c>
       <c r="P5" s="12" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="Q5" s="12" t="s">
         <v>40</v>
@@ -1724,9 +1957,9 @@
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="12" t="s">
@@ -1739,7 +1972,7 @@
         <v>32</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="G6" s="12" t="s">
         <v>9</v>
@@ -1770,10 +2003,10 @@
         <v>1</v>
       </c>
       <c r="P6" s="12" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="Q6" s="12" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="R6" s="12"/>
       <c r="S6" s="12"/>
@@ -1796,7 +2029,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
         <v>30</v>
       </c>
@@ -1868,7 +2101,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
         <v>35</v>
       </c>
@@ -1940,7 +2173,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
         <v>37</v>
       </c>
@@ -2012,9 +2245,9 @@
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13" t="s">
@@ -2084,7 +2317,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
         <v>30</v>
       </c>
@@ -2156,7 +2389,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
         <v>35</v>
       </c>
@@ -2228,7 +2461,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
         <v>37</v>
       </c>
@@ -2300,9 +2533,9 @@
         <v>109</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B14" s="14"/>
       <c r="C14" s="14" t="s">
@@ -2372,7 +2605,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>131</v>
       </c>
@@ -2427,7 +2660,7 @@
         <v>48</v>
       </c>
       <c r="S15" s="9" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="T15" s="9"/>
       <c r="U15" s="9"/>
@@ -2442,7 +2675,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>132</v>
       </c>
@@ -2497,7 +2730,7 @@
         <v>48</v>
       </c>
       <c r="S16" s="9" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="T16" s="9"/>
       <c r="U16" s="9"/>
@@ -2512,7 +2745,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>125</v>
       </c>
@@ -2567,7 +2800,7 @@
         <v>51</v>
       </c>
       <c r="S17" s="8" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="T17" s="8"/>
       <c r="U17" s="8"/>
@@ -2582,7 +2815,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>126</v>
       </c>
@@ -2637,7 +2870,7 @@
         <v>51</v>
       </c>
       <c r="S18" s="8" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="T18" s="8"/>
       <c r="U18" s="8"/>
@@ -2652,7 +2885,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>133</v>
       </c>
@@ -2718,7 +2951,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>134</v>
       </c>
@@ -2784,7 +3017,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>135</v>
       </c>
@@ -2801,7 +3034,7 @@
         <v>53</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="G21" s="7" t="s">
         <v>9</v>
@@ -2850,7 +3083,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
         <v>136</v>
       </c>
@@ -2918,7 +3151,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>91</v>
       </c>
@@ -2990,7 +3223,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>92</v>
       </c>
@@ -3062,7 +3295,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>93</v>
       </c>
@@ -3134,7 +3367,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>82</v>
       </c>
@@ -3146,13 +3379,13 @@
         <v>9</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>9</v>
@@ -3198,7 +3431,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>130</v>
       </c>
@@ -3215,7 +3448,7 @@
         <v>32</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="G27" s="6" t="s">
         <v>9</v>
@@ -3264,7 +3497,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>127</v>
       </c>
@@ -3330,7 +3563,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A29" s="10" t="s">
         <v>128</v>
       </c>
@@ -3396,7 +3629,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A30" s="10" t="s">
         <v>129</v>
       </c>
@@ -3462,9 +3695,9 @@
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B31" s="9" t="s">
         <v>117</v>
@@ -3532,9 +3765,9 @@
         <v>65</v>
       </c>
     </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B32" s="9" t="s">
         <v>117</v>
@@ -3602,13 +3835,13 @@
         <v>65</v>
       </c>
     </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>90</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D33" s="7" t="s">
         <v>9</v>
@@ -3673,13 +3906,13 @@
         <v>Three Ford Fastest Lap Compare</v>
       </c>
     </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>90</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D34" s="7" t="s">
         <v>9</v>
@@ -3744,7 +3977,7 @@
         <v>Three Ford Fastest Lap Compare</v>
       </c>
     </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
         <v>121</v>
       </c>
@@ -3814,7 +4047,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
         <v>122</v>
       </c>
@@ -3885,7 +4118,7 @@
         <v>Tyre IGL</v>
       </c>
     </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A37" s="11" t="s">
         <v>123</v>
       </c>
@@ -3956,7 +4189,7 @@
         <v>Tyre IGL</v>
       </c>
     </row>
-    <row r="38" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A38" s="11" t="s">
         <v>124</v>
       </c>
@@ -4027,7 +4260,7 @@
         <v>Tyre IGL</v>
       </c>
     </row>
-    <row r="39" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
         <v>125</v>
       </c>
@@ -4097,7 +4330,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A40" s="8" t="s">
         <v>126</v>
       </c>
@@ -4167,7 +4400,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>137</v>
       </c>
@@ -4219,10 +4452,10 @@
         <v>18</v>
       </c>
       <c r="R41" s="6" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="S41" s="6" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="T41" s="6"/>
       <c r="U41" s="6"/>
@@ -4237,7 +4470,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="42" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>138</v>
       </c>
@@ -4289,10 +4522,10 @@
         <v>56</v>
       </c>
       <c r="R42" s="6" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="S42" s="6" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="T42" s="6"/>
       <c r="U42" s="6"/>
@@ -4307,7 +4540,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>139</v>
       </c>
@@ -4359,10 +4592,10 @@
         <v>71</v>
       </c>
       <c r="R43" s="6" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="S43" s="6" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="T43" s="6"/>
       <c r="U43" s="6"/>
@@ -4377,7 +4610,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>113</v>
       </c>
@@ -4443,15 +4676,15 @@
         <v>69</v>
       </c>
     </row>
-    <row r="45" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B45" s="9" t="s">
         <v>117</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D45" s="9" t="s">
         <v>9</v>
@@ -4460,7 +4693,7 @@
         <v>141</v>
       </c>
       <c r="F45" s="9" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="G45" s="9" t="str">
         <f t="shared" ref="G45:G65" si="3">IF(ISBLANK($A45), "", G$2)</f>
@@ -4506,7 +4739,7 @@
         <v>142</v>
       </c>
       <c r="S45" s="9" t="s">
-        <v>143</v>
+        <v>179</v>
       </c>
       <c r="T45" s="9"/>
       <c r="U45" s="9"/>
@@ -4521,15 +4754,15 @@
         <v>107</v>
       </c>
     </row>
-    <row r="46" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B46" s="9" t="s">
         <v>117</v>
       </c>
       <c r="C46" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D46" s="9" t="s">
         <v>9</v>
@@ -4538,7 +4771,7 @@
         <v>141</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G46" s="9" t="str">
         <f t="shared" si="3"/>
@@ -4584,7 +4817,7 @@
         <v>142</v>
       </c>
       <c r="S46" s="9" t="s">
-        <v>143</v>
+        <v>179</v>
       </c>
       <c r="T46" s="9"/>
       <c r="U46" s="9"/>
@@ -4599,15 +4832,15 @@
         <v>107</v>
       </c>
     </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B47" s="9" t="s">
         <v>117</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D47" s="9" t="s">
         <v>9</v>
@@ -4616,7 +4849,7 @@
         <v>141</v>
       </c>
       <c r="F47" s="9" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="G47" s="9" t="str">
         <f t="shared" si="3"/>
@@ -4662,7 +4895,7 @@
         <v>142</v>
       </c>
       <c r="S47" s="9" t="s">
-        <v>144</v>
+        <v>179</v>
       </c>
       <c r="T47" s="9"/>
       <c r="U47" s="9"/>
@@ -4677,15 +4910,15 @@
         <v>107</v>
       </c>
     </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B48" s="9" t="s">
         <v>117</v>
       </c>
       <c r="C48" s="9" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D48" s="9" t="s">
         <v>9</v>
@@ -4694,7 +4927,7 @@
         <v>141</v>
       </c>
       <c r="F48" s="9" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G48" s="9" t="str">
         <f t="shared" si="3"/>
@@ -4740,7 +4973,7 @@
         <v>142</v>
       </c>
       <c r="S48" s="9" t="s">
-        <v>144</v>
+        <v>179</v>
       </c>
       <c r="T48" s="9"/>
       <c r="U48" s="9"/>
@@ -4755,15 +4988,15 @@
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A49" s="15" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B49" s="15" t="s">
         <v>117</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D49" s="15" t="s">
         <v>9</v>
@@ -4772,7 +5005,7 @@
         <v>141</v>
       </c>
       <c r="F49" s="15" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="G49" s="15" t="str">
         <f t="shared" si="3"/>
@@ -4818,7 +5051,7 @@
         <v>142</v>
       </c>
       <c r="S49" s="15" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="T49" s="15"/>
       <c r="U49" s="15"/>
@@ -4833,15 +5066,15 @@
         <v>108</v>
       </c>
     </row>
-    <row r="50" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B50" s="15" t="s">
         <v>117</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D50" s="15" t="s">
         <v>9</v>
@@ -4850,7 +5083,7 @@
         <v>141</v>
       </c>
       <c r="F50" s="15" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G50" s="15" t="str">
         <f t="shared" si="3"/>
@@ -4896,7 +5129,7 @@
         <v>142</v>
       </c>
       <c r="S50" s="15" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="T50" s="15"/>
       <c r="U50" s="15"/>
@@ -4911,15 +5144,15 @@
         <v>108</v>
       </c>
     </row>
-    <row r="51" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A51" s="15" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B51" s="15" t="s">
         <v>117</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D51" s="15" t="s">
         <v>9</v>
@@ -4928,7 +5161,7 @@
         <v>141</v>
       </c>
       <c r="F51" s="15" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="G51" s="15" t="str">
         <f t="shared" si="3"/>
@@ -4974,7 +5207,7 @@
         <v>142</v>
       </c>
       <c r="S51" s="15" t="s">
-        <v>151</v>
+        <v>179</v>
       </c>
       <c r="T51" s="15"/>
       <c r="U51" s="15"/>
@@ -4989,15 +5222,15 @@
         <v>108</v>
       </c>
     </row>
-    <row r="52" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>117</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D52" s="15" t="s">
         <v>9</v>
@@ -5006,7 +5239,7 @@
         <v>141</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G52" s="15" t="str">
         <f t="shared" si="3"/>
@@ -5052,7 +5285,7 @@
         <v>142</v>
       </c>
       <c r="S52" s="15" t="s">
-        <v>152</v>
+        <v>179</v>
       </c>
       <c r="T52" s="15"/>
       <c r="U52" s="15"/>
@@ -5067,15 +5300,15 @@
         <v>108</v>
       </c>
     </row>
-    <row r="53" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B53" s="8" t="s">
         <v>117</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D53" s="8" t="s">
         <v>9</v>
@@ -5084,7 +5317,7 @@
         <v>141</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="G53" s="8" t="str">
         <f t="shared" si="3"/>
@@ -5130,7 +5363,7 @@
         <v>142</v>
       </c>
       <c r="S53" s="8" t="s">
-        <v>143</v>
+        <v>179</v>
       </c>
       <c r="T53" s="8"/>
       <c r="U53" s="8"/>
@@ -5145,15 +5378,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="54" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A54" s="8" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B54" s="8" t="s">
         <v>117</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D54" s="8" t="s">
         <v>9</v>
@@ -5162,7 +5395,7 @@
         <v>141</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G54" s="8" t="str">
         <f t="shared" si="3"/>
@@ -5208,7 +5441,7 @@
         <v>142</v>
       </c>
       <c r="S54" s="8" t="s">
-        <v>143</v>
+        <v>179</v>
       </c>
       <c r="T54" s="8"/>
       <c r="U54" s="8"/>
@@ -5223,15 +5456,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="55" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B55" s="8" t="s">
         <v>117</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D55" s="8" t="s">
         <v>9</v>
@@ -5240,7 +5473,7 @@
         <v>141</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="G55" s="8" t="str">
         <f t="shared" si="3"/>
@@ -5286,7 +5519,7 @@
         <v>142</v>
       </c>
       <c r="S55" s="8" t="s">
-        <v>144</v>
+        <v>179</v>
       </c>
       <c r="T55" s="8"/>
       <c r="U55" s="8"/>
@@ -5301,15 +5534,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="56" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A56" s="8" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B56" s="8" t="s">
         <v>117</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>9</v>
@@ -5318,7 +5551,7 @@
         <v>141</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G56" s="8" t="str">
         <f t="shared" si="3"/>
@@ -5364,7 +5597,7 @@
         <v>142</v>
       </c>
       <c r="S56" s="8" t="s">
-        <v>144</v>
+        <v>179</v>
       </c>
       <c r="T56" s="8"/>
       <c r="U56" s="8"/>
@@ -5379,15 +5612,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="57" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B57" s="16" t="s">
         <v>117</v>
       </c>
       <c r="C57" s="16" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D57" s="16" t="s">
         <v>9</v>
@@ -5396,7 +5629,7 @@
         <v>141</v>
       </c>
       <c r="F57" s="16" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="G57" s="16" t="str">
         <f t="shared" si="3"/>
@@ -5442,7 +5675,7 @@
         <v>142</v>
       </c>
       <c r="S57" s="16" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="T57" s="16"/>
       <c r="U57" s="16"/>
@@ -5457,15 +5690,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="58" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="B58" s="16" t="s">
         <v>117</v>
       </c>
       <c r="C58" s="16" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D58" s="16" t="s">
         <v>9</v>
@@ -5474,7 +5707,7 @@
         <v>141</v>
       </c>
       <c r="F58" s="16" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G58" s="16" t="str">
         <f t="shared" si="3"/>
@@ -5520,7 +5753,7 @@
         <v>142</v>
       </c>
       <c r="S58" s="16" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="T58" s="16"/>
       <c r="U58" s="16"/>
@@ -5535,15 +5768,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="59" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="B59" s="16" t="s">
         <v>117</v>
       </c>
       <c r="C59" s="16" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D59" s="16" t="s">
         <v>9</v>
@@ -5552,7 +5785,7 @@
         <v>141</v>
       </c>
       <c r="F59" s="16" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="G59" s="16" t="str">
         <f t="shared" si="3"/>
@@ -5598,7 +5831,7 @@
         <v>142</v>
       </c>
       <c r="S59" s="16" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="T59" s="16"/>
       <c r="U59" s="16"/>
@@ -5613,15 +5846,15 @@
         <v>109</v>
       </c>
     </row>
-    <row r="60" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="B60" s="16" t="s">
         <v>117</v>
       </c>
       <c r="C60" s="16" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D60" s="16" t="s">
         <v>9</v>
@@ -5630,7 +5863,7 @@
         <v>141</v>
       </c>
       <c r="F60" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G60" s="16" t="str">
         <f t="shared" si="3"/>
@@ -5676,7 +5909,7 @@
         <v>142</v>
       </c>
       <c r="S60" s="16" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="T60" s="16"/>
       <c r="U60" s="16"/>
@@ -5691,24 +5924,24 @@
         <v>109</v>
       </c>
     </row>
-    <row r="61" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A61" s="17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B61" s="17" t="s">
         <v>117</v>
       </c>
       <c r="C61" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D61" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E61" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F61" s="17" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="G61" s="17" t="str">
         <f t="shared" si="3"/>
@@ -5765,24 +5998,24 @@
         <v>109</v>
       </c>
     </row>
-    <row r="62" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A62" s="17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B62" s="17" t="s">
         <v>117</v>
       </c>
       <c r="C62" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D62" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E62" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F62" s="17" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="G62" s="17" t="str">
         <f t="shared" si="3"/>
@@ -5839,24 +6072,24 @@
         <v>109</v>
       </c>
     </row>
-    <row r="63" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A63" s="17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B63" s="17" t="s">
         <v>117</v>
       </c>
       <c r="C63" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D63" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E63" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F63" s="17" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="G63" s="17" t="str">
         <f t="shared" si="3"/>
@@ -5913,24 +6146,24 @@
         <v>109</v>
       </c>
     </row>
-    <row r="64" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A64" s="17" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B64" s="17" t="s">
         <v>117</v>
       </c>
       <c r="C64" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D64" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E64" s="17" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F64" s="17" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G64" s="17" t="str">
         <f t="shared" si="3"/>
@@ -5987,24 +6220,24 @@
         <v>109</v>
       </c>
     </row>
-    <row r="65" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A65" s="17" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B65" s="17" t="s">
         <v>117</v>
       </c>
       <c r="C65" s="17" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D65" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E65" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="F65" s="17" t="s">
         <v>149</v>
-      </c>
-      <c r="F65" s="17" t="s">
-        <v>154</v>
       </c>
       <c r="G65" s="17" t="str">
         <f t="shared" si="3"/>
@@ -6061,9 +6294,9 @@
         <v>109</v>
       </c>
     </row>
-    <row r="66" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B66" s="6" t="s">
         <v>117</v>
@@ -6078,7 +6311,7 @@
         <v>53</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="G66" s="6" t="s">
         <v>9</v>
@@ -6106,8 +6339,8 @@
         <f t="shared" ref="O66" si="5">IF(TRIM(Q65)=TRIM(P65), O65+1, O65)</f>
         <v>23</v>
       </c>
-      <c r="P66" s="6" t="s">
-        <v>71</v>
+      <c r="P66" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="Q66" s="6" t="s">
         <v>18</v>
@@ -6124,12 +6357,12 @@
       <c r="AA66" s="6"/>
       <c r="AB66" s="6"/>
       <c r="AC66" s="6" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="67" spans="1:29" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="67" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B67" s="6" t="s">
         <v>117</v>
@@ -6140,7 +6373,7 @@
         <v>53</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="G67" s="6" t="s">
         <v>9</v>
@@ -6166,13 +6399,13 @@
       <c r="N67" s="6"/>
       <c r="O67" s="6">
         <f t="shared" ref="O67" si="6">IF(TRIM(Q66)=TRIM(P66), O66+1, O66)</f>
-        <v>23</v>
-      </c>
-      <c r="P67" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q67" s="6" t="s">
-        <v>56</v>
+        <v>24</v>
+      </c>
+      <c r="P67" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q67" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="R67" s="6"/>
       <c r="S67" s="6"/>
@@ -6186,12 +6419,12 @@
       <c r="AA67" s="6"/>
       <c r="AB67" s="6"/>
       <c r="AC67" s="6" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="68" spans="1:29" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="68" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="B68" s="6" t="s">
         <v>117</v>
@@ -6202,7 +6435,7 @@
         <v>53</v>
       </c>
       <c r="F68" s="6" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="G68" s="6" t="s">
         <v>9</v>
@@ -6228,13 +6461,13 @@
       <c r="N68" s="6"/>
       <c r="O68" s="6">
         <f t="shared" ref="O68" si="7">IF(TRIM(Q67)=TRIM(P67), O67+1, O67)</f>
-        <v>23</v>
-      </c>
-      <c r="P68" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="Q68" s="6" t="s">
-        <v>71</v>
+        <v>25</v>
+      </c>
+      <c r="P68" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q68" s="17" t="s">
+        <v>18</v>
       </c>
       <c r="R68" s="6"/>
       <c r="S68" s="6"/>
@@ -6248,7 +6481,69 @@
       <c r="AA68" s="6"/>
       <c r="AB68" s="6"/>
       <c r="AC68" s="6" t="s">
-        <v>179</v>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="69" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A69" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C69" s="6"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="G69" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H69" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="I69" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J69" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K69" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="L69" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="M69" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="N69" s="6"/>
+      <c r="O69" s="6">
+        <f t="shared" ref="O69" si="8">IF(TRIM(Q68)=TRIM(P68), O68+1, O68)</f>
+        <v>26</v>
+      </c>
+      <c r="P69" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q69" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="R69" s="6"/>
+      <c r="S69" s="6"/>
+      <c r="T69" s="6"/>
+      <c r="U69" s="6"/>
+      <c r="V69" s="6"/>
+      <c r="W69" s="6"/>
+      <c r="X69" s="6"/>
+      <c r="Y69" s="6"/>
+      <c r="Z69" s="6"/>
+      <c r="AA69" s="6"/>
+      <c r="AB69" s="6"/>
+      <c r="AC69" s="6" t="s">
+        <v>174</v>
       </c>
     </row>
   </sheetData>
@@ -6262,44 +6557,44 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD683F2B-5507-41D2-9076-F6A98DB035D6}">
   <dimension ref="G11:G18"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="11" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G11" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G12" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G13" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="14" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G14" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G15" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G16" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G17" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="7:7" x14ac:dyDescent="0.25">
       <c r="G18" s="7" t="s">
         <v>60</v>
       </c>

</xml_diff>